<commit_message>
docs: add 85% RTP model spreadsheet + overview; refresh 97% docs
Each RTP model now has its own reviewer package, generated from the current par
sheet so labels (re-themed: White Hat, Straw Pig, Horseshoe, Brick Pig, Wood
Pig) and numbers are accurate and consistent:

- Big_Bad_Wolf_Saloon_Math_Model_85%_RTP.xlsx + _Overview_85%_RTP.docx — the new
  Lean model: scaled pays (e.g. Yellow Hat 1.57/6.28/31.42), scaled bonus awards
  (brick 6.43–38.79, 128× jackpot), and its measured metrics (RTP 85.25%, base
  43.46% / bonus 41.80%, σ 8.11, max win 1,082×, avg bonus 75.1×).
- Refreshed the 97% .xlsx/.docx with the current symbol labels and figures.

Both workbooks keep live Excel formulas (totals, landing probabilities, award
expectations), recalc on open, and were checked for zero formula errors. Both
docs open with a "How the math was verified" summary and note the companion
model + the RNG/max-win caveats.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Big_Bad_Wolf_Saloon_Math_Model_97%_RTP.xlsx
+++ b/docs/Big_Bad_Wolf_Saloon_Math_Model_97%_RTP.xlsx
@@ -33,7 +33,7 @@
     <numFmt numFmtId="169" formatCode="0%;0%;&quot;-&quot;"/>
     <numFmt numFmtId="170" formatCode="0.00%;0.00%;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,13 +45,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="002E5B28"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00555555"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -63,7 +63,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -88,12 +87,6 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00888888"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="002E5B28"/>
-      <sz val="15"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -127,9 +120,6 @@
     <font>
       <name val="Arial"/>
       <color rgb="00999999"/>
-    </font>
-    <font>
-      <name val="Arial"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -239,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -282,31 +272,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -315,41 +301,41 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -731,21 +717,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BIG BAD WOLF SALOON — Math Model</t>
+          <t>BIG BAD WOLF SALOON — Math Model (Standard, 97% RTP)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>5×3 video slot · 243 ways · Theoretical RTP ≈ 97%</t>
+          <t>5×3 video slot · 243 ways · "Standard" math model · win-magnitude scale 1× vs canonical</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Spec v1.0 · 2026-05-30 · build 6df4eab · figures: tools/sim.js Monte Carlo, 50,000,000 spins @ $1</t>
+          <t>Build cefc206 · figures: tools/sim.js Monte Carlo, 50,000,000 spins @ $1 (BBW_RTP_MODEL=standard)</t>
         </is>
       </c>
     </row>
@@ -777,7 +763,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Base + Bonus; target 97%. ±0.13% (1σ) at 50M spins</t>
+          <t>Base + Bonus; target 97%</t>
         </is>
       </c>
     </row>
@@ -792,7 +778,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>243-ways line wins (~30%) + expanding wild (~19%)</t>
+          <t>243-ways line wins + expanding wild</t>
         </is>
       </c>
     </row>
@@ -818,7 +804,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.0301</v>
+        <v>0.03010000000000002</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
@@ -869,7 +855,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>6 initial + retriggers (+1 per 3+ hats)</t>
+          <t>6 initial + retriggers</t>
         </is>
       </c>
     </row>
@@ -920,7 +906,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Largest win in 50M spins (×stake)</t>
+          <t>Largest win in sim (×stake)</t>
         </is>
       </c>
       <c r="B16" s="14" t="n">
@@ -928,7 +914,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>no hard max-win cap implemented</t>
+          <t>no hard max-win cap</t>
         </is>
       </c>
     </row>
@@ -982,7 +968,7 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>All blue values are Monte-Carlo measurements (tools/sim.js). See the "Read me" sheet for how the math was verified.</t>
+          <t>This workbook documents the "Standard" model. The game also ships a Lean 85% model — same reels/feature, win sizes scaled. See the matching workbook.</t>
         </is>
       </c>
       <c r="B21" s="16" t="n"/>
@@ -1002,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1010,95 +996,105 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>How the math was verified</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1"/>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+    <row r="3" ht="56" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>1. Single source of truth</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>The pay table, reel strips and bonus rules live in src/math/par-sheet.js; the win evaluation and bonus play-through live in src/math/mathcore.js. The live game AND the verifier import the SAME files, so what is tested is exactly what players get.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>2. Monte-Carlo verifier</t>
-        </is>
-      </c>
-      <c r="B5" s="20" t="inlineStr">
-        <is>
-          <t>tools/sim.js plays N independent spins through the real evaluation code and reports RTP (base/bonus/total), hit frequency, trigger rate, volatility, per-symbol contribution and bonus-buy pricing. Headline figures here are a 50,000,000-spin run (standard error of the total ≈ 0.13%, 1σ). Repeated 10–50M runs land in 96.3%–97.2%, consistent with a true ~97%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>3. Accounting matches the game</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>A spin with 6+ hats triggers the bonus and pays the BONUS ONLY (its base line wins are forfeited, exactly as the live game does). The verifier models this, so the reported base RTP is what players actually receive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>4. Cross-checks</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>(a) Base game can be EXACTLY enumerated — only 36,729,792 equally-likely screens — to confirm base RTP to full precision. (b) Bonus expectation cross-checks against the closed-form per-tier award means on the "Bonus Awards" sheet. (c) The in-game 🧮 MATH and 📊 SIM panels run the same mathcore.js and agree within Monte-Carlo noise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>5. Reproduce</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>Run:  node tools/sim.js 50000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1"/>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Pay table, reel strips and bonus rules live in src/math/par-sheet.js; evaluation and the bonus play-through live in src/math/mathcore.js. The live game AND the verifier import the SAME files, so what is tested is exactly what players get.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="56" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>2. Selectable model</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>The "Standard" model keeps the SAME reels, trigger rate, hit frequency and volatility shape as the other model, and scales every win magnitude (line pays + bonus awards) by 1×. The scale is applied once at load (browser: localStorage; verifier: BBW_RTP_MODEL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>3. Monte-Carlo verifier</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>tools/sim.js plays 50,000,000 independent spins through the real code and reports RTP, hit frequency, trigger rate, volatility and per-symbol contribution. Total RTP standard error ≈ 0.13% (1σ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>4. Faithful accounting</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>A 6+-hat spin triggers the bonus and pays the BONUS ONLY (its base line wins are forfeited, as the live game does). The verifier models this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="56" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>5. Cross-checks</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Base game can be EXACTLY enumerated (36,729,792 equally-likely screens). Bonus expectation cross-checks against the closed-form per-tier award means (Bonus Awards sheet). In-game MATH/SIM panels run the same mathcore.js.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>6. Reproduce</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Run:  BBW_RTP_MODEL=standard node tools/sim.js 50000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>RNG NOTE</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>The reference build uses Math.random(). This is NOT a certified RNG and must be replaced with a GLI-certified RNG before real-money play. The math model is RNG-agnostic (assumes independent uniform draws), so a certified RNG does not change any figure here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>The reference build uses Math.random(). NOT a certified RNG — replace with a GLI-certified RNG before real-money play. The model is RNG-agnostic (assumes independent uniform draws), so this does not change any figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>MAX WIN NOTE</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>No max-win cap is implemented. Largest observed in 50M spins was 1,274× stake; the theoretical maximum is far higher. Specify/add a cap if a jurisdiction requires one.</t>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>No max-win cap is implemented. Largest observed was 1,274× stake; the theoretical maximum is higher. Specify a cap if a jurisdiction requires one.</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1126,14 +1122,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Paytable — per-way multiple of total stake</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Paytable (Standard) — per-way multiple of total stake</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Win for a symbol = (ways) × (pay for the span) × (stake). Ways = product of the symbols occurrences on each covered reel.</t>
         </is>
@@ -1177,7 +1173,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="22" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -1185,7 +1181,7 @@
           <t>Yellow Hat</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>hat-yellow</t>
         </is>
@@ -1195,26 +1191,26 @@
           <t>High + Scatter</t>
         </is>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="24" t="n">
         <v>1.78</v>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F5" s="24" t="n">
         <v>7.14</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="24" t="n">
         <v>35.7</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="22" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Green Hat</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
+          <t>White Hat</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>hat-green</t>
         </is>
@@ -1224,18 +1220,18 @@
           <t>Mid + Scatter</t>
         </is>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="24" t="n">
         <v>0.89</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="24" t="n">
         <v>3.57</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="24" t="n">
         <v>17.85</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
+      <c r="A7" s="22" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1243,7 +1239,7 @@
           <t>Red Hat</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>hat-red</t>
         </is>
@@ -1253,26 +1249,26 @@
           <t>Mid + Scatter</t>
         </is>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="24" t="n">
         <v>0.71</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="24" t="n">
         <v>2.86</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="24" t="n">
         <v>14.28</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
+      <c r="A8" s="22" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Suit Pig</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
+          <t>Straw Pig</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>pig-suit</t>
         </is>
@@ -1282,26 +1278,26 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="24" t="n">
         <v>1.43</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="24" t="n">
         <v>5.36</v>
       </c>
-      <c r="G8" s="25" t="n">
+      <c r="G8" s="24" t="n">
         <v>26.52</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="22" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Builder Pig</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
+          <t>Horseshoe</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>pig-contractor</t>
         </is>
@@ -1311,26 +1307,26 @@
           <t>High</t>
         </is>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="24" t="n">
         <v>1.07</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="24" t="n">
         <v>4.28</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="24" t="n">
         <v>21.42</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="22" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Shotglass</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
+          <t>Brick Pig</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>pig-nature</t>
         </is>
@@ -1340,26 +1336,26 @@
           <t>Mid</t>
         </is>
       </c>
-      <c r="E10" s="25" t="n">
+      <c r="E10" s="24" t="n">
         <v>0.71</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="24" t="n">
         <v>2.86</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="G10" s="24" t="n">
         <v>14.28</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
+      <c r="A11" s="22" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Toolbox</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
+          <t>Wood Pig</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>toolbox</t>
         </is>
@@ -1369,18 +1365,18 @@
           <t>Mid</t>
         </is>
       </c>
-      <c r="E11" s="25" t="n">
+      <c r="E11" s="24" t="n">
         <v>0.61</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="24" t="n">
         <v>2.5</v>
       </c>
-      <c r="G11" s="25" t="n">
+      <c r="G11" s="24" t="n">
         <v>12.24</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="22" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1388,7 +1384,7 @@
           <t>Wolf</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>wolf</t>
         </is>
@@ -1398,18 +1394,18 @@
           <t>Low-mid</t>
         </is>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="E12" s="24" t="n">
         <v>0.46</v>
       </c>
-      <c r="F12" s="25" t="n">
+      <c r="F12" s="24" t="n">
         <v>1.79</v>
       </c>
-      <c r="G12" s="25" t="n">
+      <c r="G12" s="24" t="n">
         <v>8.67</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
+      <c r="A13" s="22" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1417,7 +1413,7 @@
           <t>Buzzard</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>buzzard</t>
         </is>
@@ -1427,213 +1423,197 @@
           <t>Low-mid</t>
         </is>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E13" s="24" t="n">
         <v>0.36</v>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" s="24" t="n">
         <v>1.43</v>
       </c>
-      <c r="G13" s="25" t="n">
+      <c r="G13" s="24" t="n">
         <v>7.14</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n">
+      <c r="A14" s="22" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
+          <t>Wolf Wild</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Wild (substitutes; no pay)</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
           <t>Ace</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>royal-a</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Royal</t>
         </is>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E15" s="24" t="n">
         <v>0.26</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F15" s="24" t="n">
         <v>0.89</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G15" s="24" t="n">
         <v>4.46</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>King</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C16" s="23" t="inlineStr">
         <is>
           <t>royal-k</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Royal</t>
         </is>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E16" s="24" t="n">
         <v>0.26</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F16" s="24" t="n">
         <v>0.89</v>
       </c>
-      <c r="G15" s="25" t="n">
+      <c r="G16" s="24" t="n">
         <v>4.46</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Queen</t>
         </is>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>royal-q</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Royal</t>
         </is>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E17" s="24" t="n">
         <v>0.21</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F17" s="24" t="n">
         <v>0.71</v>
       </c>
-      <c r="G16" s="25" t="n">
+      <c r="G17" s="24" t="n">
         <v>3.57</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="23" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Jack</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>royal-j</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Royal</t>
         </is>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E18" s="24" t="n">
         <v>0.21</v>
       </c>
-      <c r="F17" s="25" t="n">
+      <c r="F18" s="24" t="n">
         <v>0.71</v>
       </c>
-      <c r="G17" s="25" t="n">
+      <c r="G18" s="24" t="n">
         <v>3.57</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="23" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Ten</t>
         </is>
       </c>
-      <c r="C18" s="24" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>royal-10</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Royal</t>
         </is>
       </c>
-      <c r="E18" s="25" t="n">
+      <c r="E19" s="24" t="n">
         <v>0.18</v>
       </c>
-      <c r="F18" s="25" t="n">
+      <c r="F19" s="24" t="n">
         <v>0.54</v>
       </c>
-      <c r="G18" s="25" t="n">
+      <c r="G19" s="24" t="n">
         <v>2.68</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Wolf Wild</t>
-        </is>
-      </c>
-      <c r="C19" s="24" t="inlineStr">
-        <is>
-          <t>wild</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Wild (substitutes; no pay)</t>
-        </is>
-      </c>
-      <c r="E19" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Hard Hats pay as ways AND act as the bonus scatter. Wilds substitute for all except hats. Pays are 0.51× an earlier revision (see Read me).</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
-      <c r="G21" s="17" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A21:G21"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1644,7 +1624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1657,9 +1637,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Reel composition (counts per reel)</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Reel composition (counts per reel) — identical across models</t>
         </is>
       </c>
     </row>
@@ -1706,45 +1686,45 @@
           <t>Yellow Hat</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="27" t="n">
+      <c r="C4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="27" t="n">
+      <c r="D4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="27" t="n">
+      <c r="E4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="28" t="n"/>
+      <c r="G4" s="22" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Green Hat</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="n">
+          <t>White Hat</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="28" t="n"/>
+      <c r="G5" s="22" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1752,114 +1732,114 @@
           <t>Red Hat</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="28" t="n"/>
+      <c r="G6" s="22" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Suit Pig</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="n">
+          <t>Straw Pig</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="28" t="n"/>
+      <c r="G7" s="22" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Builder Pig</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="n">
+          <t>Horseshoe</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="28" t="n"/>
+      <c r="G8" s="22" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Shotglass</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="n">
+          <t>Brick Pig</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="28" t="n"/>
+      <c r="G9" s="22" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Toolbox</t>
-        </is>
-      </c>
-      <c r="B10" s="27" t="n">
+          <t>Wood Pig</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="28" t="n"/>
+      <c r="G10" s="22" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1867,22 +1847,22 @@
           <t>Wolf</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="28" t="n"/>
+      <c r="G11" s="22" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1890,22 +1870,22 @@
           <t>Buzzard</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="28" t="n"/>
+      <c r="G12" s="22" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1913,22 +1893,22 @@
           <t>Wolf Wild</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
+      <c r="B13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="28" t="n"/>
+      <c r="G13" s="22" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1936,22 +1916,22 @@
           <t>Ace</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
+      <c r="B14" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="27" t="n">
+      <c r="C14" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="27" t="n">
+      <c r="D14" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="27" t="n">
+      <c r="E14" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="G14" s="28" t="n"/>
+      <c r="G14" s="22" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1959,22 +1939,22 @@
           <t>King</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
+      <c r="B15" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="27" t="n">
+      <c r="E15" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="28" t="n"/>
+      <c r="G15" s="22" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1982,22 +1962,22 @@
           <t>Queen</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
+      <c r="B16" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="27" t="n">
+      <c r="D16" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="28" t="n"/>
+      <c r="G16" s="22" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -2005,22 +1985,22 @@
           <t>Jack</t>
         </is>
       </c>
-      <c r="B17" s="27" t="n">
+      <c r="B17" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="C17" s="27" t="n">
+      <c r="C17" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="27" t="n">
+      <c r="D17" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="27" t="n">
+      <c r="E17" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="27" t="n">
+      <c r="F17" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="G17" s="28" t="n"/>
+      <c r="G17" s="22" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -2028,66 +2008,50 @@
           <t>Ten</t>
         </is>
       </c>
-      <c r="B18" s="27" t="n">
+      <c r="B18" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="C18" s="27" t="n">
+      <c r="C18" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="27" t="n">
+      <c r="D18" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="E18" s="27" t="n">
+      <c r="E18" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="G18" s="28" t="n"/>
+      <c r="G18" s="22" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Strip length</t>
         </is>
       </c>
-      <c r="B19" s="30" t="n"/>
-      <c r="C19" s="30" t="n"/>
-      <c r="D19" s="30" t="n"/>
-      <c r="E19" s="30" t="n"/>
-      <c r="F19" s="30" t="n"/>
-      <c r="G19" s="30" t="n"/>
+      <c r="B19" s="28" t="n"/>
+      <c r="C19" s="28" t="n"/>
+      <c r="D19" s="28" t="n"/>
+      <c r="E19" s="28" t="n"/>
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>Hats (all 3)</t>
         </is>
       </c>
-      <c r="B20" s="30" t="n"/>
-      <c r="C20" s="30" t="n"/>
-      <c r="D20" s="30" t="n"/>
-      <c r="E20" s="30" t="n"/>
-      <c r="F20" s="30" t="n"/>
-      <c r="G20" s="30" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Blue = input counts. Black = formulas. Outcome space = product of strip lengths = 36,729,792 equally-likely screens. Hats ≈ 9.2% of positions → ~1/179 trigger.</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
-      <c r="G22" s="17" t="n"/>
+      <c r="B20" s="28" t="n"/>
+      <c r="C20" s="28" t="n"/>
+      <c r="D20" s="28" t="n"/>
+      <c r="E20" s="28" t="n"/>
+      <c r="F20" s="28" t="n"/>
+      <c r="G20" s="28" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A22:G22"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2098,7 +2062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2110,247 +2074,225 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Expected occurrences per reel window  =  3 × count ÷ strip length</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Mean number of cells of each symbol in a reels 3-cell window (the colCount the ways math consumes). For single-copy symbols this equals P(present).</t>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>R5</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>R5</t>
-        </is>
-      </c>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Yellow Hat</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="n"/>
+      <c r="C4" s="29" t="n"/>
+      <c r="D4" s="29" t="n"/>
+      <c r="E4" s="29" t="n"/>
+      <c r="F4" s="29" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Yellow Hat</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="n"/>
-      <c r="C5" s="31" t="n"/>
-      <c r="D5" s="31" t="n"/>
-      <c r="E5" s="31" t="n"/>
-      <c r="F5" s="31" t="n"/>
+          <t>White Hat</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="n"/>
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="29" t="n"/>
+      <c r="E5" s="29" t="n"/>
+      <c r="F5" s="29" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Green Hat</t>
-        </is>
-      </c>
-      <c r="B6" s="31" t="n"/>
-      <c r="C6" s="31" t="n"/>
-      <c r="D6" s="31" t="n"/>
-      <c r="E6" s="31" t="n"/>
-      <c r="F6" s="31" t="n"/>
+          <t>Red Hat</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="n"/>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="29" t="n"/>
+      <c r="E6" s="29" t="n"/>
+      <c r="F6" s="29" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Red Hat</t>
-        </is>
-      </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
-      <c r="E7" s="31" t="n"/>
-      <c r="F7" s="31" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Straw Pig</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="29" t="n"/>
+      <c r="F7" s="29" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Suit Pig</t>
-        </is>
-      </c>
-      <c r="B8" s="31" t="n"/>
-      <c r="C8" s="31" t="n"/>
-      <c r="D8" s="31" t="n"/>
-      <c r="E8" s="31" t="n"/>
-      <c r="F8" s="31" t="n"/>
+          <t>Horseshoe</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="29" t="n"/>
+      <c r="F8" s="29" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Builder Pig</t>
-        </is>
-      </c>
-      <c r="B9" s="31" t="n"/>
-      <c r="C9" s="31" t="n"/>
-      <c r="D9" s="31" t="n"/>
-      <c r="E9" s="31" t="n"/>
-      <c r="F9" s="31" t="n"/>
+          <t>Brick Pig</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="29" t="n"/>
+      <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Shotglass</t>
-        </is>
-      </c>
-      <c r="B10" s="31" t="n"/>
-      <c r="C10" s="31" t="n"/>
-      <c r="D10" s="31" t="n"/>
-      <c r="E10" s="31" t="n"/>
-      <c r="F10" s="31" t="n"/>
+          <t>Wood Pig</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n"/>
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="29" t="n"/>
+      <c r="F10" s="29" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Toolbox</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="31" t="n"/>
-      <c r="D11" s="31" t="n"/>
-      <c r="E11" s="31" t="n"/>
-      <c r="F11" s="31" t="n"/>
+          <t>Wolf</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="n"/>
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n"/>
+      <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Wolf</t>
-        </is>
-      </c>
-      <c r="B12" s="31" t="n"/>
-      <c r="C12" s="31" t="n"/>
-      <c r="D12" s="31" t="n"/>
-      <c r="E12" s="31" t="n"/>
-      <c r="F12" s="31" t="n"/>
+          <t>Buzzard</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="29" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Buzzard</t>
-        </is>
-      </c>
-      <c r="B13" s="31" t="n"/>
-      <c r="C13" s="31" t="n"/>
-      <c r="D13" s="31" t="n"/>
-      <c r="E13" s="31" t="n"/>
-      <c r="F13" s="31" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Wolf Wild</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="29" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Wolf Wild</t>
-        </is>
-      </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
-      <c r="E14" s="31" t="n"/>
-      <c r="F14" s="31" t="n"/>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Ace</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n"/>
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="n"/>
+      <c r="F14" s="29" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Ace</t>
-        </is>
-      </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="31" t="n"/>
-      <c r="E15" s="31" t="n"/>
-      <c r="F15" s="31" t="n"/>
+          <t>King</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="n"/>
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="29" t="n"/>
+      <c r="F15" s="29" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>King</t>
-        </is>
-      </c>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="31" t="n"/>
-      <c r="E16" s="31" t="n"/>
-      <c r="F16" s="31" t="n"/>
+          <t>Queen</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n"/>
+      <c r="C16" s="29" t="n"/>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="29" t="n"/>
+      <c r="F16" s="29" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Queen</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="31" t="n"/>
-      <c r="E17" s="31" t="n"/>
-      <c r="F17" s="31" t="n"/>
+          <t>Jack</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="n"/>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="29" t="n"/>
+      <c r="F17" s="29" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Jack</t>
-        </is>
-      </c>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="31" t="n"/>
-      <c r="D18" s="31" t="n"/>
-      <c r="E18" s="31" t="n"/>
-      <c r="F18" s="31" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
           <t>Ten</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="31" t="n"/>
-      <c r="E19" s="31" t="n"/>
-      <c r="F19" s="31" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Green = links to the Reel Counts sheet (live; updates if counts change).</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="17" t="n"/>
+      <c r="B18" s="29" t="n"/>
+      <c r="C18" s="29" t="n"/>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="29" t="n"/>
+      <c r="F18" s="29" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A21:F21"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2373,16 +2315,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Physical reel strips (exact order)</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Physical reel strips (exact order) — identical across models</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="32" t="inlineStr">
-        <is>
-          <t>Legend: HY/HG/HR=Yellow/Green/Red Hat · PS=Suit Pig · PC=Builder Pig · PN=Shotglass · TB=Toolbox · WF=Wolf · BZ=Buzzard · A/K/Q/J/10=Royals · WILD=Wolf Wild</t>
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Legend: HY=Yellow Hat · HG=White Hat · HR=Red Hat · PS=Straw Pig · PC=Horseshoe · PN=Brick Pig · TB=Wood Pig · WF=Wolf · BZ=Buzzard · A/K/Q/J/10=Royals · WILD=Wolf Wild</t>
         </is>
       </c>
     </row>
@@ -2419,996 +2361,996 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="33" t="n">
+      <c r="A5" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="E5" s="23" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="F5" s="23" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="n">
+      <c r="A6" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="E6" s="23" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="F6" s="23" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="n">
+      <c r="A7" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
-      <c r="F7" s="23" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="n">
+      <c r="A8" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="n">
+      <c r="A9" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="F9" s="23" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="n">
+      <c r="A10" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>BZ</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>BZ</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>BZ</t>
         </is>
       </c>
-      <c r="E10" s="23" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>BZ</t>
         </is>
       </c>
-      <c r="F10" s="23" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
         <is>
           <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="n">
+      <c r="A11" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D11" s="34" t="inlineStr">
+      <c r="D11" s="32" t="inlineStr">
         <is>
           <t>WILD</t>
         </is>
       </c>
-      <c r="E11" s="23" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F11" s="23" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="n">
+      <c r="A12" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="F12" s="23" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="n">
+      <c r="A13" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E13" s="23" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="F13" s="23" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="n">
+      <c r="A14" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C14" s="35" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>HY</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="F14" s="23" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="n">
+      <c r="A15" s="31" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B15" s="33" t="inlineStr">
         <is>
           <t>HY</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>HG</t>
         </is>
       </c>
-      <c r="D15" s="35" t="inlineStr">
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>HY</t>
         </is>
       </c>
-      <c r="E15" s="35" t="inlineStr">
+      <c r="E15" s="33" t="inlineStr">
         <is>
           <t>HY</t>
         </is>
       </c>
-      <c r="F15" s="23" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="n">
+      <c r="A16" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="35" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>HY</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="D16" s="35" t="inlineStr">
+      <c r="D16" s="33" t="inlineStr">
         <is>
           <t>HG</t>
         </is>
       </c>
-      <c r="E16" s="35" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>HG</t>
         </is>
       </c>
-      <c r="F16" s="23" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="33" t="n">
+      <c r="A17" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F17" s="23" t="inlineStr">
+      <c r="F17" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="33" t="n">
+      <c r="A18" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E18" s="23" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="F18" s="23" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="n">
+      <c r="A19" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="E19" s="23" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="F19" s="35" t="inlineStr">
+      <c r="F19" s="33" t="inlineStr">
         <is>
           <t>HY</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="33" t="n">
+      <c r="A20" s="31" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>WF</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E20" s="23" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F20" s="35" t="inlineStr">
+      <c r="F20" s="33" t="inlineStr">
         <is>
           <t>HG</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="33" t="n">
+      <c r="A21" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E21" s="23" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="F21" s="23" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="33" t="n">
+      <c r="A22" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="E22" s="23" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="F22" s="23" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="33" t="n">
+      <c r="A23" s="31" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E23" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="F23" s="23" t="inlineStr">
+      <c r="F23" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="33" t="n">
+      <c r="A24" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F24" s="23" t="inlineStr">
+      <c r="F24" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="33" t="n">
+      <c r="A25" s="31" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C25" s="35" t="inlineStr">
+      <c r="C25" s="33" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
+      <c r="D25" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E25" s="23" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F25" s="23" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="33" t="n">
+      <c r="A26" s="31" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="B26" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E26" s="23" t="inlineStr">
+      <c r="E26" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="F26" s="23" t="inlineStr">
+      <c r="F26" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="33" t="n">
+      <c r="A27" s="31" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="35" t="inlineStr">
+      <c r="B27" s="33" t="inlineStr">
         <is>
           <t>HG</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D27" s="35" t="inlineStr">
+      <c r="D27" s="33" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="E27" s="35" t="inlineStr">
+      <c r="E27" s="33" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="F27" s="23" t="inlineStr">
+      <c r="F27" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="33" t="n">
+      <c r="A28" s="31" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="35" t="inlineStr">
+      <c r="B28" s="33" t="inlineStr">
         <is>
           <t>HR</t>
         </is>
       </c>
-      <c r="C28" s="23" t="inlineStr">
+      <c r="C28" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="D28" s="23" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="E28" s="23" t="inlineStr">
+      <c r="E28" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="F28" s="23" t="inlineStr">
+      <c r="F28" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="n">
+      <c r="A29" s="31" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="23" t="inlineStr">
+      <c r="B29" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="C29" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="D29" s="23" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="E29" s="23" t="inlineStr">
+      <c r="E29" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="F29" s="23" t="inlineStr">
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="33" t="n">
+      <c r="A30" s="31" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="23" t="inlineStr">
+      <c r="B30" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C30" s="23" t="inlineStr">
+      <c r="C30" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="D30" s="23" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E30" s="23" t="inlineStr">
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F30" s="23" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="33" t="n">
+      <c r="A31" s="31" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C31" s="23" t="inlineStr">
+      <c r="C31" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E31" s="23" t="inlineStr">
+      <c r="E31" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F31" s="23" t="inlineStr">
+      <c r="F31" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="33" t="n">
+      <c r="A32" s="31" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B32" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
+      <c r="C32" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D32" s="23" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E32" s="23" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="F32" s="23" t="inlineStr">
+      <c r="F32" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="33" t="n">
+      <c r="A33" s="31" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B33" s="22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="D33" s="23" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="E33" s="23" t="inlineStr">
+      <c r="E33" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="F33" s="23" t="inlineStr">
+      <c r="F33" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="33" t="n">
+      <c r="A34" s="31" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="23" t="inlineStr">
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C34" s="23" t="inlineStr">
+      <c r="C34" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="D34" s="23" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="E34" s="23" t="inlineStr">
+      <c r="E34" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="F34" s="23" t="inlineStr">
+      <c r="F34" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="33" t="n">
+      <c r="A35" s="31" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B35" s="22" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C35" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="D35" s="23" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E35" s="23" t="inlineStr">
+      <c r="E35" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F35" s="23" t="inlineStr">
+      <c r="F35" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="33" t="n">
+      <c r="A36" s="31" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="B36" s="22" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C36" s="23" t="inlineStr">
+      <c r="C36" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D36" s="23" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E36" s="23" t="inlineStr">
+      <c r="E36" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F36" s="23" t="n"/>
+      <c r="F36" s="22" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="33" t="n">
+      <c r="A37" s="31" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="B37" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="inlineStr">
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E37" s="23" t="inlineStr">
+      <c r="E37" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F37" s="23" t="n"/>
+      <c r="F37" s="22" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="33" t="n">
+      <c r="A38" s="31" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="23" t="inlineStr">
+      <c r="B38" s="22" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
+      <c r="F38" s="22" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3434,16 +3376,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Hard Hat Free Spins — award math</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Hard Hat Free Spins — award math (Standard)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Each built house pays once when the wolf blows it down (wolf reveal). Awards in × stake. U(a,b)=uniform on [a,b].</t>
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Each built house pays once when the wolf blows it down. Awards in × stake. U(a,b)=uniform on [a,b].</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3427,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3495,22 +3437,22 @@
           <t>🏚️ Straw</t>
         </is>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="24" t="n">
         <v>0.46</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="24" t="n">
         <v>2.44</v>
       </c>
-      <c r="E5" s="37" t="n">
+      <c r="E5" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="38" t="n"/>
+      <c r="G5" s="36" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3520,22 +3462,22 @@
           <t>🏠 Stick</t>
         </is>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="24" t="n">
         <v>2.44</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="24" t="n">
         <v>9.74</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="E6" s="35" t="n">
         <v>0.04</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="26" t="n">
         <v>29</v>
       </c>
-      <c r="G6" s="38" t="n"/>
+      <c r="G6" s="36" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="34" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -3545,22 +3487,22 @@
           <t>🏰 Brick</t>
         </is>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="24" t="n">
         <v>7.31</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="24" t="n">
         <v>44.08</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="E7" s="35" t="n">
         <v>0.04</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="26" t="n">
         <v>146</v>
       </c>
-      <c r="G7" s="38" t="n"/>
+      <c r="G7" s="36" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="39" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Mansion Jackpot</t>
         </is>
@@ -3595,7 +3537,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>E[award | fire] formula</t>
+          <t>E[award|fire]</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -3615,25 +3557,25 @@
           <t>3+ brick houses &amp; a fresh brick</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n">
+      <c r="B11" s="38" t="n">
         <v>24.4</v>
       </c>
-      <c r="C11" s="40" t="n">
+      <c r="C11" s="38" t="n">
         <v>19.7</v>
       </c>
-      <c r="D11" s="41" t="n">
+      <c r="D11" s="39" t="n">
         <v>3</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>base + perBrick×bricks/2</t>
-        </is>
-      </c>
-      <c r="F11" s="42" t="n"/>
-      <c r="G11" s="42" t="n"/>
+          <t>base+perBrick×bricks/2</t>
+        </is>
+      </c>
+      <c r="F11" s="40" t="n"/>
+      <c r="G11" s="40" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="39" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t>Feature structure &amp; Bonus Buy</t>
         </is>
@@ -3687,7 +3629,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>3+ hats in a spin → +1 free spin</t>
+          <t>3+ hats → +1 free spin</t>
         </is>
       </c>
       <c r="C16" s="16" t="n"/>
@@ -3704,7 +3646,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>each hat upgrades its cell: straw → stick → brick (persistent, max tier 3)</t>
+          <t>each hat upgrades its cell: straw → stick → brick (max tier 3)</t>
         </is>
       </c>
       <c r="C17" s="16" t="n"/>
@@ -3721,7 +3663,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>paid normally during the feature (same paytable, wild active)</t>
+          <t>paid normally during the feature</t>
         </is>
       </c>
       <c r="C18" s="16" t="n"/>
@@ -3755,7 +3697,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>88 × stake  →  buy RTP = 85.47/88 ≈ 97.1% ≈ game RTP</t>
+          <t>88 × stake → buy RTP ≈ 97.1% ≈ game RTP</t>
         </is>
       </c>
       <c r="C20" s="16" t="n"/>
@@ -3767,9 +3709,9 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B16:G16"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B17:G17"/>
@@ -3786,7 +3728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3794,16 +3736,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Base-game RTP contribution by symbol</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Base-game RTP contribution by symbol (Standard)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Share of total stake returned by each symbol in the base game (20M-spin run). Wild reads 0% (no own pay) — its value shows up inside the symbols it extends, chiefly the royals.</t>
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Share of total stake returned by each symbol in the base game. Wild reads 0% (no own pay) — its value shows up inside the symbols it extends, chiefly the royals.</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3767,7 @@
           <t>Ten</t>
         </is>
       </c>
-      <c r="B5" s="43" t="n">
+      <c r="B5" s="41" t="n">
         <v>0.1515</v>
       </c>
     </row>
@@ -3835,7 +3777,7 @@
           <t>King</t>
         </is>
       </c>
-      <c r="B6" s="43" t="n">
+      <c r="B6" s="41" t="n">
         <v>0.0794</v>
       </c>
     </row>
@@ -3845,7 +3787,7 @@
           <t>Ace</t>
         </is>
       </c>
-      <c r="B7" s="43" t="n">
+      <c r="B7" s="41" t="n">
         <v>0.07539999999999999</v>
       </c>
     </row>
@@ -3855,7 +3797,7 @@
           <t>Jack</t>
         </is>
       </c>
-      <c r="B8" s="43" t="n">
+      <c r="B8" s="41" t="n">
         <v>0.0667</v>
       </c>
     </row>
@@ -3865,17 +3807,17 @@
           <t>Queen</t>
         </is>
       </c>
-      <c r="B9" s="43" t="n">
+      <c r="B9" s="41" t="n">
         <v>0.0667</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Toolbox</t>
-        </is>
-      </c>
-      <c r="B10" s="43" t="n">
+          <t>Wood Pig</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="n">
         <v>0.0134</v>
       </c>
     </row>
@@ -3885,37 +3827,37 @@
           <t>Wolf</t>
         </is>
       </c>
-      <c r="B11" s="43" t="n">
+      <c r="B11" s="41" t="n">
         <v>0.0132</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Suit Pig</t>
-        </is>
-      </c>
-      <c r="B12" s="43" t="n">
+          <t>Straw Pig</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="n">
         <v>0.0119</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Builder Pig</t>
-        </is>
-      </c>
-      <c r="B13" s="43" t="n">
+          <t>Horseshoe</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="n">
         <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Shotglass</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="n">
+          <t>Brick Pig</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="n">
         <v>0.003</v>
       </c>
     </row>
@@ -3925,7 +3867,7 @@
           <t>Yellow Hat</t>
         </is>
       </c>
-      <c r="B15" s="43" t="n">
+      <c r="B15" s="41" t="n">
         <v>0.0015</v>
       </c>
     </row>
@@ -3935,7 +3877,7 @@
           <t>Buzzard</t>
         </is>
       </c>
-      <c r="B16" s="43" t="n">
+      <c r="B16" s="41" t="n">
         <v>0.0013</v>
       </c>
     </row>
@@ -3945,17 +3887,17 @@
           <t>Red Hat</t>
         </is>
       </c>
-      <c r="B17" s="43" t="n">
+      <c r="B17" s="41" t="n">
         <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Green Hat</t>
-        </is>
-      </c>
-      <c r="B18" s="43" t="n">
+          <t>White Hat</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="n">
         <v>0.0004</v>
       </c>
     </row>
@@ -3965,30 +3907,19 @@
           <t>Wolf Wild</t>
         </is>
       </c>
-      <c r="B19" s="43" t="n">
+      <c r="B19" s="41" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>BASE GAME TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="44" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Royals lead because reel 3 (which expands) carries the most royals; their ways extend through the wild reel. This is the expanding wilds contribution, distributed across the substituted symbols.</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="n"/>
+      <c r="B20" s="42" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A22:B22"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3999,16 +3930,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Configuration constants</t>
         </is>
@@ -4027,211 +3958,228 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Source (par-sheet.js)</t>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Reels × rows</t>
-        </is>
-      </c>
-      <c r="B4" s="41" t="inlineStr">
-        <is>
-          <t>5 × 3</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>REEL_COUNT, ROWS_PER_REEL</t>
+          <t>RTP model</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>Standard (standard)</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>RTP_MODELS</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Ways</t>
-        </is>
-      </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>243</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>derived (3^5, left-to-right)</t>
+          <t>Win-magnitude scale</t>
+        </is>
+      </c>
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t>1×</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>RTP_MODELS[].scale</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Minimum win span</t>
-        </is>
-      </c>
-      <c r="B6" s="41" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>MIN_WIN_SPAN</t>
+          <t>Reels × rows</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>5 × 3</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>REEL_COUNT, ROWS_PER_REEL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Bonus trigger hats</t>
-        </is>
-      </c>
-      <c r="B7" s="41" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>BONUS_TRIGGER_HATS</t>
+          <t>Ways</t>
+        </is>
+      </c>
+      <c r="B7" s="39" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>derived</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Initial free spins</t>
-        </is>
-      </c>
-      <c r="B8" s="41" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>FREE_SPINS_INITIAL</t>
+          <t>Minimum win span</t>
+        </is>
+      </c>
+      <c r="B8" s="39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>MIN_WIN_SPAN</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Retrigger hats / award</t>
-        </is>
-      </c>
-      <c r="B9" s="41" t="inlineStr">
-        <is>
-          <t>3 / +1</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>RETRIGGER_HATS, retriggerSpins</t>
+          <t>Bonus trigger hats</t>
+        </is>
+      </c>
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>BONUS_TRIGGER_HATS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Max house tier</t>
-        </is>
-      </c>
-      <c r="B10" s="41" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>MAX_FRAME_TIER</t>
+          <t>Initial free spins</t>
+        </is>
+      </c>
+      <c r="B10" s="39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>FREE_SPINS_INITIAL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Tier-2/3 jackpot chance</t>
-        </is>
-      </c>
-      <c r="B11" s="41" t="inlineStr">
-        <is>
-          <t>4% / 4%</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>BONUS_CONFIG.tiers</t>
+          <t>Retrigger hats / award</t>
+        </is>
+      </c>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>3 / +1</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>RETRIGGER_HATS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Mansion min bricks / base / per-brick</t>
-        </is>
-      </c>
-      <c r="B12" s="41" t="inlineStr">
-        <is>
-          <t>3 / 24.4 / 19.7</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>BONUS_CONFIG.mansion</t>
+          <t>Max house tier</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>MAX_FRAME_TIER</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Bonus-Buy multiplier</t>
-        </is>
-      </c>
-      <c r="B13" s="41" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>BONUS_CONFIG.buyCostMult</t>
+          <t>Tier-2/3 jackpot chance</t>
+        </is>
+      </c>
+      <c r="B13" s="39" t="inlineStr">
+        <is>
+          <t>4% / 4%</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>BONUS_CONFIG.tiers</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Stake levels</t>
-        </is>
-      </c>
-      <c r="B14" s="41" t="inlineStr">
-        <is>
-          <t>0.20, 0.50, 1, 2, 5, 10, 20, 50</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="inlineStr">
-        <is>
-          <t>BET_LEVELS</t>
+          <t>Mansion min bricks / base / per-brick</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>3 / 24.4 / 19.7</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>BONUS_CONFIG.mansion</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Default stake / balance</t>
-        </is>
-      </c>
-      <c r="B15" s="41" t="inlineStr">
-        <is>
-          <t>1.00 / 1000.00</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>DEFAULT_BET_INDEX, DEFAULT_BALANCE</t>
+          <t>Bonus-Buy multiplier</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>BONUS_CONFIG.buyCostMult</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Stake levels</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>0.20 … 50.00</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>BET_LEVELS</t>
         </is>
       </c>
     </row>

</xml_diff>